<commit_message>
actualiza readme, fusiona los bunkers de laredo, y actualiza archivos excel en inventory_by-bunkers
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventory_by_bunker/BUNKER 2954 Saltillo.xlsx
+++ b/inventory_by_bunker/BUNKER 2954 Saltillo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Bunker de Refacciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B5B9E3F-3271-4601-8647-E1A3FC9DFBE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E5047A3-3D62-46D6-85E3-667DA9C52173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{1CB12F25-FA39-4960-A9AD-DD44B8374742}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="147">
   <si>
     <t>Cantidad</t>
   </si>
@@ -59,9 +59,6 @@
     <t>Nombre</t>
   </si>
   <si>
-    <t>Descripción</t>
-  </si>
-  <si>
     <t>Fabricante</t>
   </si>
   <si>
@@ -71,27 +68,12 @@
     <t>Serie</t>
   </si>
   <si>
-    <t>Condición</t>
-  </si>
-  <si>
-    <t>impresora termica</t>
-  </si>
-  <si>
-    <t>impresora</t>
-  </si>
-  <si>
-    <t>epson</t>
-  </si>
-  <si>
     <t>TM-T88VI</t>
   </si>
   <si>
     <t>X9XN014561</t>
   </si>
   <si>
-    <t>Reparado</t>
-  </si>
-  <si>
     <t>TM-T70II</t>
   </si>
   <si>
@@ -140,9 +122,6 @@
     <t>X9XQ029793</t>
   </si>
   <si>
-    <t>impresora laser</t>
-  </si>
-  <si>
     <t xml:space="preserve">HP </t>
   </si>
   <si>
@@ -158,9 +137,6 @@
     <t>PHBTT14240</t>
   </si>
   <si>
-    <t>Impresora portatil</t>
-  </si>
-  <si>
     <t>zebra</t>
   </si>
   <si>
@@ -173,72 +149,18 @@
     <t>AC3FA4D8A7D2</t>
   </si>
   <si>
-    <t>Buje</t>
-  </si>
-  <si>
-    <t>Buje de etiquetas</t>
-  </si>
-  <si>
-    <t>Bizerva</t>
-  </si>
-  <si>
     <t>N/A</t>
   </si>
   <si>
-    <t xml:space="preserve">seguro </t>
-  </si>
-  <si>
-    <t>seguro de guarda de etiqueta</t>
-  </si>
-  <si>
-    <t>Buje recolector</t>
-  </si>
-  <si>
-    <t>orejas de buje de etiquetas</t>
-  </si>
-  <si>
-    <t>potenciometro de radio</t>
-  </si>
-  <si>
-    <t>motorola</t>
-  </si>
-  <si>
-    <t>dep450</t>
-  </si>
-  <si>
     <t>Nuevo</t>
   </si>
   <si>
-    <t>USB de datos para bascula</t>
-  </si>
-  <si>
     <t>Datalogic</t>
   </si>
   <si>
-    <t>magallane 9800I</t>
-  </si>
-  <si>
-    <t>USB de datos para pinpad</t>
-  </si>
-  <si>
-    <t>ingenico</t>
-  </si>
-  <si>
-    <t>lane 7000</t>
-  </si>
-  <si>
-    <t>power inyector</t>
-  </si>
-  <si>
     <t>Cisco</t>
   </si>
   <si>
-    <t>air-pwrinj6</t>
-  </si>
-  <si>
-    <t>Gomas Pick roller bandeja 1</t>
-  </si>
-  <si>
     <t>M806</t>
   </si>
   <si>
@@ -251,9 +173,6 @@
     <t>S120E05808</t>
   </si>
   <si>
-    <t>contactos de media vuleta</t>
-  </si>
-  <si>
     <t>F400E022376</t>
   </si>
   <si>
@@ -269,96 +188,36 @@
     <t>X9XN014857</t>
   </si>
   <si>
-    <t>carro Bizerva</t>
-  </si>
-  <si>
-    <t>bizerva</t>
-  </si>
-  <si>
     <t>AC3FA480EE68</t>
   </si>
   <si>
     <t>AC3FA4DC03BE</t>
   </si>
   <si>
-    <t>telefono analogo</t>
-  </si>
-  <si>
-    <t>panasonic</t>
-  </si>
-  <si>
     <t>kx-ts550me</t>
   </si>
   <si>
-    <t>%5EAFK006654</t>
-  </si>
-  <si>
-    <t>caja hermetica</t>
-  </si>
-  <si>
-    <t>contacto hembra media vuelta</t>
-  </si>
-  <si>
-    <t>clavija de media vuleta</t>
-  </si>
-  <si>
     <t>TDR</t>
   </si>
   <si>
     <t>G18HE9592</t>
   </si>
   <si>
-    <t>cpu</t>
-  </si>
-  <si>
-    <t>dell</t>
-  </si>
-  <si>
-    <t>optiplex 3070</t>
-  </si>
-  <si>
     <t>BQ76H13</t>
   </si>
   <si>
-    <t>Thinclient</t>
-  </si>
-  <si>
     <t>8CN11000X2</t>
   </si>
   <si>
-    <t>JP</t>
-  </si>
-  <si>
     <t>NO VISIBLE</t>
   </si>
   <si>
-    <t>verificador</t>
-  </si>
-  <si>
-    <t>varificador</t>
-  </si>
-  <si>
-    <t>mk319</t>
-  </si>
-  <si>
     <t>S18129522501238</t>
   </si>
   <si>
-    <t>fusor 506</t>
-  </si>
-  <si>
-    <t>teclado POS</t>
-  </si>
-  <si>
-    <t>prehkeytec</t>
-  </si>
-  <si>
     <t>mci 128</t>
   </si>
   <si>
-    <t>bascula toledo</t>
-  </si>
-  <si>
     <t>Toledo</t>
   </si>
   <si>
@@ -368,12 +227,6 @@
     <t>B541554102</t>
   </si>
   <si>
-    <t>bascula datalogic</t>
-  </si>
-  <si>
-    <t>datalogic</t>
-  </si>
-  <si>
     <t>F17H09267</t>
   </si>
   <si>
@@ -383,18 +236,9 @@
     <t>F18I11783</t>
   </si>
   <si>
-    <t>filminas 806</t>
-  </si>
-  <si>
     <t>m806</t>
   </si>
   <si>
-    <t>rodillos de trasferencia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">monitor </t>
-  </si>
-  <si>
     <t>V193</t>
   </si>
   <si>
@@ -434,18 +278,6 @@
     <t>6CM7061D0D</t>
   </si>
   <si>
-    <t xml:space="preserve"> bascula</t>
-  </si>
-  <si>
-    <t>bascula</t>
-  </si>
-  <si>
-    <t>XC115E modular</t>
-  </si>
-  <si>
-    <t xml:space="preserve">falta carrito de impresión, touch no funciona </t>
-  </si>
-  <si>
     <t>3CQ61429B5</t>
   </si>
   <si>
@@ -458,15 +290,6 @@
     <t>P5TF148161</t>
   </si>
   <si>
-    <t>escaner de mano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">escaner de mano </t>
-  </si>
-  <si>
-    <t>gd4400</t>
-  </si>
-  <si>
     <t>F16D07854</t>
   </si>
   <si>
@@ -477,13 +300,205 @@
   </si>
   <si>
     <t>F14L00190</t>
+  </si>
+  <si>
+    <t>Epson</t>
+  </si>
+  <si>
+    <t>Impresora</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zebra </t>
+  </si>
+  <si>
+    <t>Zebra</t>
+  </si>
+  <si>
+    <t>Condicion</t>
+  </si>
+  <si>
+    <t>Descripcion</t>
+  </si>
+  <si>
+    <t>Impresora Termica</t>
+  </si>
+  <si>
+    <t>Impresora Laser</t>
+  </si>
+  <si>
+    <t>Impresora Portatil</t>
+  </si>
+  <si>
+    <t>Bizerba</t>
+  </si>
+  <si>
+    <t>Motorola</t>
+  </si>
+  <si>
+    <t>DEP 450</t>
+  </si>
+  <si>
+    <t>Magellan 9800I</t>
+  </si>
+  <si>
+    <t>Ingenico</t>
+  </si>
+  <si>
+    <t>Cable PinPad</t>
+  </si>
+  <si>
+    <t>Cable Datos</t>
+  </si>
+  <si>
+    <t>Power Injector</t>
+  </si>
+  <si>
+    <t>Lane 7000</t>
+  </si>
+  <si>
+    <t>Air-pwrinj6</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>Gomas Pick Roller</t>
+  </si>
+  <si>
+    <t>Contacto de Seguridad</t>
+  </si>
+  <si>
+    <t>Nema L5-15</t>
+  </si>
+  <si>
+    <t>Bryant</t>
+  </si>
+  <si>
+    <t>Impresor Bizerba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bascula </t>
+  </si>
+  <si>
+    <t>Telefono Analogo</t>
+  </si>
+  <si>
+    <t>Caja Hermetica</t>
+  </si>
+  <si>
+    <t>Panduit</t>
+  </si>
+  <si>
+    <t>Panasonic</t>
+  </si>
+  <si>
+    <t>5EAFK006654</t>
+  </si>
+  <si>
+    <t>Clavija de Seguridad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clavija de Seguridad </t>
+  </si>
+  <si>
+    <t>Eaton</t>
+  </si>
+  <si>
+    <t>Desktop</t>
+  </si>
+  <si>
+    <t>CPU</t>
+  </si>
+  <si>
+    <t>Optiplex 3070</t>
+  </si>
+  <si>
+    <t>Thin Client</t>
+  </si>
+  <si>
+    <t>T640</t>
+  </si>
+  <si>
+    <t>HP</t>
+  </si>
+  <si>
+    <t>Verificador de Precios</t>
+  </si>
+  <si>
+    <t>MK319</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fusor </t>
+  </si>
+  <si>
+    <t>Fusor</t>
+  </si>
+  <si>
+    <t>Teclado POS</t>
+  </si>
+  <si>
+    <t>PrehKeyTec</t>
+  </si>
+  <si>
+    <t>MCI 128</t>
+  </si>
+  <si>
+    <t>Bascula Etiquetadora</t>
+  </si>
+  <si>
+    <t>Bascula</t>
+  </si>
+  <si>
+    <t>Bascula / Escaner</t>
+  </si>
+  <si>
+    <t>Filmina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rodillos de Transferencia </t>
+  </si>
+  <si>
+    <t>Rodillos de Transferencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monitor </t>
+  </si>
+  <si>
+    <t xml:space="preserve">XC115E </t>
+  </si>
+  <si>
+    <t>Escaner Manual</t>
+  </si>
+  <si>
+    <t>GD4400</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buje </t>
+  </si>
+  <si>
+    <t>Seguro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recolector </t>
+  </si>
+  <si>
+    <t>Orejas de Buje</t>
+  </si>
+  <si>
+    <t>Potenciometro Radio</t>
+  </si>
+  <si>
+    <t>Radiofrecuencia</t>
+  </si>
+  <si>
+    <t>Para  Refacciones</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -502,6 +517,17 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -522,12 +548,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="-0.499984740745262"/>
+        <fgColor theme="3" tint="0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -536,27 +562,18 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FFE5E7EB"/>
+      <left style="thin">
+        <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color rgb="FFE5E7EB"/>
+      <right style="thin">
+        <color indexed="64"/>
       </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFE5E7EB"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFE5E7EB"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFE5E7EB"/>
+      <top style="thin">
+        <color indexed="64"/>
       </top>
-      <bottom/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -566,13 +583,13 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1069,35 +1086,36 @@
   <dimension ref="A1:G74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.90625" style="3"/>
-    <col min="2" max="2" width="26" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.90625" style="3"/>
-    <col min="5" max="5" width="16.26953125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="14.1796875" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="41.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.90625" style="1"/>
+    <col min="2" max="2" width="26" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.6328125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.1796875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.26953125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="33.08984375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="41.453125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
       <c r="G1" s="2" t="s">
-        <v>6</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
@@ -1105,22 +1123,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>7</v>
+        <v>89</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>9</v>
+        <v>83</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -1128,22 +1146,22 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>14</v>
-      </c>
       <c r="G3" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
@@ -1151,22 +1169,22 @@
         <v>1</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>13</v>
-      </c>
       <c r="F4" s="3" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -1174,22 +1192,22 @@
         <v>1</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>13</v>
-      </c>
       <c r="F5" s="3" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -1197,22 +1215,22 @@
         <v>1</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>13</v>
-      </c>
       <c r="F6" s="3" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
@@ -1220,22 +1238,22 @@
         <v>1</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>19</v>
-      </c>
       <c r="G7" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
@@ -1243,22 +1261,22 @@
         <v>1</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>13</v>
-      </c>
       <c r="F8" s="3" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -1266,22 +1284,22 @@
         <v>1</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>7</v>
+        <v>89</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>9</v>
+        <v>83</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
@@ -1289,22 +1307,22 @@
         <v>1</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>7</v>
+        <v>89</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>9</v>
+        <v>83</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -1312,22 +1330,22 @@
         <v>1</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>7</v>
+        <v>89</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>9</v>
+        <v>83</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
@@ -1335,22 +1353,22 @@
         <v>1</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>7</v>
+        <v>89</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>9</v>
+        <v>83</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
@@ -1358,22 +1376,22 @@
         <v>1</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>7</v>
+        <v>89</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>9</v>
+        <v>83</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
@@ -1381,22 +1399,22 @@
         <v>1</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>7</v>
+        <v>89</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>9</v>
+        <v>83</v>
       </c>
       <c r="E14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F14" s="3" t="s">
-        <v>28</v>
-      </c>
       <c r="G14" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
@@ -1404,22 +1422,22 @@
         <v>1</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>29</v>
+        <v>90</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
@@ -1427,22 +1445,22 @@
         <v>1</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>29</v>
+        <v>90</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
@@ -1450,22 +1468,22 @@
         <v>1</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>35</v>
+        <v>91</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
@@ -1473,22 +1491,22 @@
         <v>1</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>35</v>
+        <v>91</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>36</v>
+        <v>86</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
@@ -1496,22 +1514,22 @@
         <v>1</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>40</v>
+        <v>140</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>41</v>
+        <v>131</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>42</v>
+        <v>92</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
@@ -1519,22 +1537,22 @@
         <v>3</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>44</v>
+        <v>141</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>45</v>
+        <v>131</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>42</v>
+        <v>92</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
@@ -1542,22 +1560,22 @@
         <v>1</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>46</v>
+        <v>142</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>46</v>
+        <v>131</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>42</v>
+        <v>92</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
@@ -1565,22 +1583,22 @@
         <v>4</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>47</v>
+        <v>143</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>47</v>
+        <v>131</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>42</v>
+        <v>92</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
@@ -1588,19 +1606,22 @@
         <v>2</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>48</v>
+        <v>144</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>48</v>
+        <v>145</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>49</v>
+        <v>93</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>50</v>
+        <v>94</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>102</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
@@ -1608,19 +1629,22 @@
         <v>1</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>52</v>
+        <v>98</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>52</v>
+        <v>98</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>54</v>
+        <v>95</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>102</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
@@ -1628,19 +1652,22 @@
         <v>4</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>55</v>
+        <v>97</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>55</v>
+        <v>97</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>57</v>
+        <v>100</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>102</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
@@ -1648,22 +1675,22 @@
         <v>1</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>58</v>
+        <v>99</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>58</v>
+        <v>99</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>59</v>
+        <v>35</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>60</v>
+        <v>101</v>
       </c>
       <c r="F26" s="3">
         <v>134158</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
@@ -1671,19 +1698,22 @@
         <v>4</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>61</v>
+        <v>103</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>61</v>
+        <v>103</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>62</v>
+        <v>36</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>102</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
@@ -1691,22 +1721,22 @@
         <v>1</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>64</v>
+        <v>38</v>
       </c>
       <c r="E28" s="3">
         <v>4500</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>65</v>
+        <v>39</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
@@ -1714,19 +1744,22 @@
         <v>3</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>66</v>
+        <v>104</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>66</v>
+        <v>104</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>106</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>43</v>
+        <v>105</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
@@ -1734,22 +1767,22 @@
         <v>1</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>64</v>
+        <v>38</v>
       </c>
       <c r="E30" s="3">
         <v>4500</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>67</v>
+        <v>40</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
@@ -1757,22 +1790,22 @@
         <v>1</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>64</v>
+        <v>38</v>
       </c>
       <c r="E31" s="3">
         <v>4500</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>68</v>
+        <v>41</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
@@ -1780,22 +1813,22 @@
         <v>1</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>64</v>
+        <v>38</v>
       </c>
       <c r="E32" s="3">
         <v>4500</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>69</v>
+        <v>42</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
@@ -1803,22 +1836,22 @@
         <v>1</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>7</v>
+        <v>89</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>9</v>
+        <v>83</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
@@ -1826,22 +1859,22 @@
         <v>1</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>7</v>
+        <v>89</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>9</v>
+        <v>83</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
@@ -1849,22 +1882,22 @@
         <v>2</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>72</v>
+        <v>107</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>72</v>
+        <v>108</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
@@ -1872,22 +1905,22 @@
         <v>1</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>35</v>
+        <v>91</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>74</v>
+        <v>45</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
@@ -1895,22 +1928,22 @@
         <v>1</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>35</v>
+        <v>91</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>75</v>
+        <v>46</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
@@ -1918,22 +1951,22 @@
         <v>1</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>76</v>
+        <v>109</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>76</v>
+        <v>109</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>77</v>
+        <v>112</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
@@ -1941,22 +1974,22 @@
         <v>3</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>80</v>
+        <v>110</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>43</v>
+        <v>110</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>43</v>
+        <v>111</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
@@ -1964,22 +1997,22 @@
         <v>3</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>43</v>
+        <v>104</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>43</v>
+        <v>106</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>43</v>
+        <v>105</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
@@ -1987,22 +2020,22 @@
         <v>1</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>82</v>
+        <v>114</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>43</v>
+        <v>115</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>43</v>
+        <v>116</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>43</v>
+        <v>105</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
@@ -2010,19 +2043,20 @@
         <v>1</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>83</v>
+        <v>48</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>83</v>
+        <v>48</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>53</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="E42" s="3"/>
       <c r="F42" s="3" t="s">
-        <v>84</v>
+        <v>49</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
@@ -2030,22 +2064,22 @@
         <v>1</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>86</v>
+        <v>64</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>87</v>
+        <v>119</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>88</v>
+        <v>50</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
@@ -2053,22 +2087,22 @@
         <v>1</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>89</v>
+        <v>120</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>89</v>
+        <v>120</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="E44" s="3">
-        <v>640</v>
+        <v>23</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>121</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>90</v>
+        <v>51</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
@@ -2076,22 +2110,22 @@
         <v>1</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>89</v>
+        <v>120</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>89</v>
+        <v>120</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="E45" s="3">
-        <v>640</v>
+        <v>122</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>121</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>92</v>
+        <v>52</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
@@ -2099,22 +2133,22 @@
         <v>1</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>93</v>
+        <v>123</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>94</v>
+        <v>123</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>36</v>
+        <v>86</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>95</v>
+        <v>124</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>96</v>
+        <v>53</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
@@ -2122,22 +2156,22 @@
         <v>1</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>97</v>
+        <v>125</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>97</v>
+        <v>126</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="E47" s="3" t="s">
-        <v>43</v>
+        <v>122</v>
+      </c>
+      <c r="E47" s="3">
+        <v>506</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
@@ -2145,22 +2179,22 @@
         <v>1</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>99</v>
+        <v>128</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>100</v>
+        <v>129</v>
       </c>
       <c r="F48" s="3">
         <v>1605954</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
@@ -2168,22 +2202,22 @@
         <v>1</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>99</v>
+        <v>128</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>100</v>
+        <v>129</v>
       </c>
       <c r="F49" s="3">
         <v>1855980</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
@@ -2191,22 +2225,22 @@
         <v>1</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>99</v>
+        <v>128</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>100</v>
+        <v>129</v>
       </c>
       <c r="F50" s="3">
         <v>1887527</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
@@ -2214,22 +2248,22 @@
         <v>1</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>101</v>
+        <v>130</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>102</v>
+        <v>55</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>103</v>
+        <v>56</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>104</v>
+        <v>57</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
@@ -2237,22 +2271,22 @@
         <v>1</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>105</v>
+        <v>132</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>105</v>
+        <v>131</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>106</v>
+        <v>34</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>54</v>
+        <v>95</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>107</v>
+        <v>58</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
@@ -2260,22 +2294,22 @@
         <v>1</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>105</v>
+        <v>132</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>105</v>
+        <v>131</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>106</v>
+        <v>34</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>54</v>
+        <v>95</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>108</v>
+        <v>59</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
@@ -2283,22 +2317,22 @@
         <v>1</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>105</v>
+        <v>132</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>105</v>
+        <v>131</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>106</v>
+        <v>34</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>54</v>
+        <v>95</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>109</v>
+        <v>60</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.35">
@@ -2306,22 +2340,22 @@
         <v>3</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>111</v>
+        <v>61</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
@@ -2329,22 +2363,22 @@
         <v>3</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>112</v>
+        <v>134</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>111</v>
+        <v>61</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
@@ -2352,22 +2386,22 @@
         <v>1</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>114</v>
+        <v>62</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>115</v>
+        <v>63</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.35">
@@ -2375,22 +2409,22 @@
         <v>1</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>116</v>
+        <v>64</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>117</v>
+        <v>65</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>118</v>
+        <v>66</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
@@ -2398,22 +2432,22 @@
         <v>1</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>119</v>
+        <v>67</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>120</v>
+        <v>68</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.35">
@@ -2421,22 +2455,22 @@
         <v>1</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>121</v>
+        <v>69</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>122</v>
+        <v>70</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.35">
@@ -2444,22 +2478,22 @@
         <v>1</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>116</v>
+        <v>64</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>123</v>
+        <v>71</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>124</v>
+        <v>72</v>
       </c>
       <c r="G61" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.35">
@@ -2467,22 +2501,22 @@
         <v>1</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>125</v>
+        <v>73</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>126</v>
+        <v>74</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.35">
@@ -2490,22 +2524,22 @@
         <v>1</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>42</v>
+        <v>92</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="F63" s="3">
         <v>20249709</v>
       </c>
       <c r="G63" s="3" t="s">
-        <v>130</v>
+        <v>146</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
@@ -2513,22 +2547,22 @@
         <v>1</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>42</v>
+        <v>92</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="F64" s="3">
         <v>20273773</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>130</v>
+        <v>146</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.35">
@@ -2536,22 +2570,22 @@
         <v>1</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>42</v>
+        <v>92</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="F65" s="3">
         <v>20378438</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>130</v>
+        <v>146</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.35">
@@ -2559,22 +2593,22 @@
         <v>1</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>119</v>
+        <v>67</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>131</v>
+        <v>75</v>
       </c>
       <c r="G66" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.35">
@@ -2582,22 +2616,22 @@
         <v>1</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>35</v>
+        <v>91</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>9</v>
+        <v>83</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>132</v>
+        <v>76</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.35">
@@ -2605,22 +2639,22 @@
         <v>1</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>35</v>
+        <v>91</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>9</v>
+        <v>83</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>133</v>
+        <v>77</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.35">
@@ -2628,22 +2662,22 @@
         <v>1</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>35</v>
+        <v>91</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>9</v>
+        <v>83</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>134</v>
+        <v>78</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.35">
@@ -2651,22 +2685,22 @@
         <v>1</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>138</v>
+        <v>79</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.35">
@@ -2674,22 +2708,22 @@
         <v>1</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>99</v>
+        <v>128</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>100</v>
+        <v>54</v>
       </c>
       <c r="F71" s="3">
         <v>1459124</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.35">
@@ -2697,22 +2731,22 @@
         <v>1</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>139</v>
+        <v>80</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.35">
@@ -2720,22 +2754,22 @@
         <v>1</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>140</v>
+        <v>81</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.35">
@@ -2743,25 +2777,26 @@
         <v>1</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>141</v>
+        <v>82</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>